<commit_message>
chore(fase-1B.8): cierre sub-fase 1B-local + xlsx test reports
Smoke API contra backend levantado + PostgreSQL real:
- 46/46 integration (auth + endpoints + repos)
- 27/27 backend domain
- 220/220 frontend unit (modo mock por default)
- 10/10 smoke curl: /auth/me x3 roles, /categories, sessions CRUD,
  IDOR 404 cross-owner, DELETE 204.

Cobertura completa del contrato camelCase (1B.7) end-to-end. Frontend
puede operar contra backend real seteando NEXT_PUBLIC_API_URL.

- Agregadas filas al `docs/test-reports/test-runs.xlsx`.
- `apps/backend/.env.example` documenta `SQA_KB_DATABASE_URL` para que
  cualquier dev levante uvicorn sin tener que adivinar el DSN.
- `IMPLEMENTATION-STATUS.md` marca 1B-local completa (1B.4 Blob y 1B.6
  LLM diferidos a Fase 2 donde se necesitan para el agente).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-reports/test-runs.xlsx
+++ b/docs/test-reports/test-runs.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="47">
   <si>
     <t>Fecha</t>
   </si>
@@ -113,6 +113,45 @@
   </si>
   <si>
     <t>Cierre Fase 1B.5 — endpoints CRUD (taxonomy + documents + sessions + dashboard)</t>
+  </si>
+  <si>
+    <t>2026-05-23 01:12:28</t>
+  </si>
+  <si>
+    <t>b687217</t>
+  </si>
+  <si>
+    <t>integration</t>
+  </si>
+  <si>
+    <t>Fase 1B.7-1B.8 backend integration (auth+endpoints+repos) contra PG real</t>
+  </si>
+  <si>
+    <t>2026-05-23 01:12:29</t>
+  </si>
+  <si>
+    <t>unit-frontend</t>
+  </si>
+  <si>
+    <t>Fase 1B.7 frontend post camelCase dispatcher (modo mock)</t>
+  </si>
+  <si>
+    <t>2026-05-23 01:12:30</t>
+  </si>
+  <si>
+    <t>unit-backend</t>
+  </si>
+  <si>
+    <t>Fase 1B.7 backend domain tests post alias_generator=to_camel</t>
+  </si>
+  <si>
+    <t>2026-05-23 01:12:45</t>
+  </si>
+  <si>
+    <t>smoke-api</t>
+  </si>
+  <si>
+    <t>Fase 1B.8 smoke curl: /auth/me x3 roles, /categories, /sessions CRUD, IDOR 404, DELETE 204</t>
   </si>
 </sst>
 </file>
@@ -498,7 +537,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="19" customWidth="1"/>
@@ -743,6 +782,122 @@
         <v>33</v>
       </c>
     </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>34</v>
+      </c>
+      <c r="B9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" t="s">
+        <v>35</v>
+      </c>
+      <c r="D9" t="s">
+        <v>36</v>
+      </c>
+      <c r="E9">
+        <v>46</v>
+      </c>
+      <c r="F9">
+        <v>46</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>8.35</v>
+      </c>
+      <c r="I9" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" t="s">
+        <v>35</v>
+      </c>
+      <c r="D10" t="s">
+        <v>39</v>
+      </c>
+      <c r="E10">
+        <v>220</v>
+      </c>
+      <c r="F10">
+        <v>220</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>17.75</v>
+      </c>
+      <c r="I10" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B11" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" t="s">
+        <v>42</v>
+      </c>
+      <c r="E11">
+        <v>27</v>
+      </c>
+      <c r="F11">
+        <v>27</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <v>0.27</v>
+      </c>
+      <c r="I11" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>44</v>
+      </c>
+      <c r="B12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" t="s">
+        <v>35</v>
+      </c>
+      <c r="D12" t="s">
+        <v>45</v>
+      </c>
+      <c r="E12">
+        <v>10</v>
+      </c>
+      <c r="F12">
+        <v>10</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>2</v>
+      </c>
+      <c r="I12" t="s">
+        <v>46</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>

<commit_message>
chore(fase-2.7): cierre Fase 2 — STATUS + xlsx test report
- IMPLEMENTATION-STATUS: tabla resumen muestra Fase 2 ✅, avance total
  ~60% (12/20 semanas-equivalentes), 9 fases cerradas. Sección Fase 2
  detallada con cobertura por componente, decisiones (modelo, checkpointer,
  buffer SSE, text-delta granularidad) y pendientes diferidos (smoke
  con Anthropic real, Blob adapter, prompt caching activación).
- xlsx: fila final 420/420 backend tests verdes.

Smoke real con Anthropic API NO ejecutado por regla del usuario — queda
para cuando confirme go-live.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-reports/test-runs.xlsx
+++ b/docs/test-reports/test-runs.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="51">
   <si>
     <t>Fecha</t>
   </si>
@@ -152,6 +152,18 @@
   </si>
   <si>
     <t>Fase 1B.8 smoke curl: /auth/me x3 roles, /categories, /sessions CRUD, IDOR 404, DELETE 204</t>
+  </si>
+  <si>
+    <t>2026-05-25 11:49:59</t>
+  </si>
+  <si>
+    <t>fase-2-agente-langgraph</t>
+  </si>
+  <si>
+    <t>9e39d0b</t>
+  </si>
+  <si>
+    <t>Fase 2 cierre — backend agente LangGraph end-to-end. Modos A/B/C + endpoint SSE con 14 eventos. 420 tests, sin tocar Anthropic real.</t>
   </si>
 </sst>
 </file>
@@ -537,7 +549,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="19" customWidth="1"/>
@@ -898,6 +910,35 @@
         <v>46</v>
       </c>
     </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>47</v>
+      </c>
+      <c r="B13" t="s">
+        <v>48</v>
+      </c>
+      <c r="C13" t="s">
+        <v>49</v>
+      </c>
+      <c r="D13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13">
+        <v>420</v>
+      </c>
+      <c r="F13">
+        <v>420</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <v>27</v>
+      </c>
+      <c r="I13" t="s">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>

<commit_message>
docs(fase-4): cierre — STATUS al 100% + fila xlsx (774 tests)
Fase 4 completa (4.0 a 4.6). Avance del proyecto ~83%. Branch
fase-4-docs listo para merge a master.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-reports/test-runs.xlsx
+++ b/docs/test-reports/test-runs.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="74">
   <si>
     <t>Fecha</t>
   </si>
@@ -221,6 +221,18 @@
   </si>
   <si>
     <t>Fase 3.7 eval rag (recall@5=1.0, precision@1=1.0). Determinista — sin Cohere real. Validacion dual con TI diferida a Fase 11.</t>
+  </si>
+  <si>
+    <t>2026-05-27 19:30:04</t>
+  </si>
+  <si>
+    <t>fase-4-docs</t>
+  </si>
+  <si>
+    <t>b96fdab</t>
+  </si>
+  <si>
+    <t>Fase 4 cierre — generacion (docx/pptx/xlsx/pdf/md) + extractores + anonimizador + endpoints /ingestion + adapter Blob Azurite + worker. +126 tests vs 648. 4 skipped (Azurite/PG condicionales).</t>
   </si>
 </sst>
 </file>
@@ -606,7 +618,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="19" customWidth="1"/>
@@ -1170,6 +1182,35 @@
         <v>69</v>
       </c>
     </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>70</v>
+      </c>
+      <c r="B20" t="s">
+        <v>71</v>
+      </c>
+      <c r="C20" t="s">
+        <v>72</v>
+      </c>
+      <c r="D20" t="s">
+        <v>21</v>
+      </c>
+      <c r="E20">
+        <v>774</v>
+      </c>
+      <c r="F20">
+        <v>774</v>
+      </c>
+      <c r="G20">
+        <v>0</v>
+      </c>
+      <c r="H20">
+        <v>49.87</v>
+      </c>
+      <c r="I20" t="s">
+        <v>73</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>